<commit_message>
Implement binary line graph
</commit_message>
<xml_diff>
--- a/20250519_ErCoIn_SA/output/20250519_ErCoIn_SA_element_pairs.xlsx
+++ b/20250519_ErCoIn_SA/output/20250519_ErCoIn_SA_element_pairs.xlsx
@@ -7,11 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Er-Co" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Co-In" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="In-In" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Er-In" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Co-Co" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Co-Co" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Er-In" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Er-Co" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Co-In" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="In-In" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -452,11 +452,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1814810.cif</t>
+          <t>1818414.cif</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2.623</v>
+        <v>2.231</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -467,44 +467,74 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1956508.cif</t>
+          <t>1234749.cif</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2.799</v>
+        <v>2.46</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Full occupancy</t>
+          <t>Full occupancy with atomic mixing</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr"/>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>1925389.cif</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2.492</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Full occupancy</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>1814810.cif</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>2.964</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Deficiency with atomic mixing</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr"/>
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
           <t>Average</t>
         </is>
       </c>
-      <c r="B5" t="n">
-        <v>2.711</v>
-      </c>
-      <c r="C5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="B7" t="n">
+        <v>2.537</v>
+      </c>
+      <c r="C7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>SD</t>
         </is>
       </c>
-      <c r="B6" t="n">
-        <v>0.124</v>
-      </c>
-      <c r="C6" t="inlineStr"/>
+      <c r="B8" t="n">
+        <v>0.308</v>
+      </c>
+      <c r="C8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -517,7 +547,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -540,59 +570,194 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1956508.cif</t>
+          <t>1234749.cif</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2.687</v>
+        <v>2.859</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Deficiency without atomic mixing</t>
+          <t>Full occupancy with atomic mixing</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1814810.cif</t>
+          <t>1634753.cif</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2.964</v>
+        <v>2.959</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Deficiency with atomic mixing</t>
+          <t>Full occupancy</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr"/>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>1818414.cif</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2.962</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Full occupancy with atomic mixing</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Average</t>
+          <t>1140826.cif</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2.826</v>
-      </c>
-      <c r="C5" t="inlineStr"/>
+        <v>2.975</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Full occupancy</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>1234747.cif</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>3.035</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Full occupancy</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>1803318.cif</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>3.051</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Full occupancy</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>1814810.cif</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>3.055</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Full occupancy with atomic mixing</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>1229705.cif</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>3.137</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Full occupancy</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>1840445.cif</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>3.174</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Full occupancy</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>1710931.cif</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>3.199</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Full occupancy</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>1920543.cif</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>3.222</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Full occupancy</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr"/>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>3.057</v>
+      </c>
+      <c r="C14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
           <t>SD</t>
         </is>
       </c>
-      <c r="B6" t="n">
-        <v>0.196</v>
-      </c>
-      <c r="C6" t="inlineStr"/>
+      <c r="B15" t="n">
+        <v>0.115</v>
+      </c>
+      <c r="C15" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -605,7 +770,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -628,11 +793,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1956508.cif</t>
+          <t>1814810.cif</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2.949</v>
+        <v>2.623</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -643,11 +808,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1814810.cif</t>
+          <t>1803318.cif</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3.009</v>
+        <v>2.644</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -656,31 +821,196 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr"/>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>1840445.cif</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2.691</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Full occupancy</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Average</t>
+          <t>1818414.cif</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2.979</v>
-      </c>
-      <c r="C5" t="inlineStr"/>
+        <v>2.729</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Full occupancy</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>1234747.cif</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>2.737</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Full occupancy</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>1140826.cif</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>2.743</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Full occupancy</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>1229705.cif</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>2.794</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Full occupancy</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>1956508.cif</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>2.799</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Full occupancy</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>1000761.cif</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>2.81</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Full occupancy</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>1234749.cif</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>2.859</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Full occupancy with atomic mixing</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>1233938.cif</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>2.881</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Full occupancy</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>1803512.cif</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>2.882</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Full occupancy</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>1925389.cif</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>2.922</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Full occupancy</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr"/>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>2.778</v>
+      </c>
+      <c r="C16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>SD</t>
         </is>
       </c>
-      <c r="B6" t="n">
-        <v>0.042</v>
-      </c>
-      <c r="C6" t="inlineStr"/>
+      <c r="B17" t="n">
+        <v>0.094</v>
+      </c>
+      <c r="C17" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -693,7 +1023,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -716,42 +1046,224 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1814810.cif</t>
+          <t>1634753.cif</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3.055</v>
+        <v>2.447</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>Full occupancy</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>1234749.cif</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2.46</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
           <t>Full occupancy with atomic mixing</t>
         </is>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr"/>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Average</t>
+          <t>1803512.cif</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3.055</v>
-      </c>
-      <c r="C4" t="inlineStr"/>
+        <v>2.618</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Full occupancy</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>1233938.cif</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>2.626</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Full occupancy</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>1956508.cif</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>2.687</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Deficiency without atomic mixing</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>1920543.cif</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>2.687</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Full occupancy</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>1710931.cif</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>2.691</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Full occupancy</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>1000761.cif</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>2.705</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Full occupancy</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>1840445.cif</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>2.813</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Full occupancy</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>1925389.cif</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>2.922</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Full occupancy</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>1229705.cif</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Full occupancy</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>1814810.cif</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>2.964</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Deficiency with atomic mixing</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>1803318.cif</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>2.975</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Full occupancy</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr"/>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>2.733</v>
+      </c>
+      <c r="C16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>SD</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr"/>
+      <c r="B17" t="n">
+        <v>0.178</v>
+      </c>
+      <c r="C17" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -764,7 +1276,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -787,42 +1299,164 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1814810.cif</t>
+          <t>1234749.cif</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2.964</v>
+        <v>2.46</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Deficiency with atomic mixing</t>
+          <t>Full occupancy with atomic mixing</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>1229705.cif</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2.926</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Full occupancy</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Average</t>
+          <t>1000761.cif</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2.964</v>
-      </c>
-      <c r="C4" t="inlineStr"/>
+        <v>2.948</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Full occupancy</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>1956508.cif</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>2.949</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Full occupancy</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>1840445.cif</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>2.967</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Full occupancy</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>1803318.cif</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>2.999</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Full occupancy</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>1814810.cif</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>3.009</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Full occupancy</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>1920543.cif</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>3.09</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Full occupancy</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>1710931.cif</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>3.199</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Full occupancy</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr"/>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>2.95</v>
+      </c>
+      <c r="C12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>SD</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr"/>
+      <c r="B13" t="n">
+        <v>0.203</v>
+      </c>
+      <c r="C13" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>